<commit_message>
Work in progress for ASCII wheel and 1500 calibration
Now to add to menu system to allow switching modes
</commit_message>
<xml_diff>
--- a/docs/wheelwriter/keyboard_matrix.xlsx
+++ b/docs/wheelwriter/keyboard_matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dave\Desktop\IBM 1620 Jr\Console Typewriter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Documents\WIP2\Cadetwriter\docs\wheelwriter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40B3D41-7E22-4943-BB08-DF8EEA7EB179}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D198297-6336-475B-87E3-215C0FAAED45}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{5E82A069-CE49-40B7-9E46-07FE8FC3DAB8}"/>
+    <workbookView xWindow="-120" yWindow="225" windowWidth="29040" windowHeight="17895" firstSheet="4" activeTab="10" xr2:uid="{5E82A069-CE49-40B7-9E46-07FE8FC3DAB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Wheelwriter 1000" sheetId="2" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="ASCII Keyboard" sheetId="10" r:id="rId8"/>
     <sheet name="IBM 1620 Max" sheetId="11" r:id="rId9"/>
     <sheet name="IBM 1620 Max Keyboard" sheetId="12" r:id="rId10"/>
+    <sheet name="Print Wheels" sheetId="15" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="6">ASCII!$A$1:$Q$13</definedName>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="443">
   <si>
     <t>KYBD-8
 J14-8</t>
@@ -6271,13 +6272,338 @@
       </rPr>
       <t>&lt;load paper&gt;</t>
     </r>
+  </si>
+  <si>
+    <t>Wheel
+Location</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>o</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>q</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>;</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>:</t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>'</t>
+  </si>
+  <si>
+    <t>"</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>!</t>
+  </si>
+  <si>
+    <t>{</t>
+  </si>
+  <si>
+    <t>}</t>
+  </si>
+  <si>
+    <t>&gt;</t>
+  </si>
+  <si>
+    <t>&lt;</t>
+  </si>
+  <si>
+    <t>~</t>
+  </si>
+  <si>
+    <t>|</t>
+  </si>
+  <si>
+    <t>\</t>
+  </si>
+  <si>
+    <t>[</t>
+  </si>
+  <si>
+    <t>]</t>
+  </si>
+  <si>
+    <t>&amp;</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>@</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>^</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>,</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>(</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>)</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>&lt;cent&gt;</t>
+  </si>
+  <si>
+    <t>+/-</t>
+  </si>
+  <si>
+    <t>&lt;sup 3&gt;</t>
+  </si>
+  <si>
+    <t>&lt;sup 2&gt;</t>
+  </si>
+  <si>
+    <t>&lt;degree&gt;</t>
+  </si>
+  <si>
+    <t>&lt;section&gt;</t>
+  </si>
+  <si>
+    <t>&lt;paragraph&gt;</t>
+  </si>
+  <si>
+    <t>1/2</t>
+  </si>
+  <si>
+    <t>1/4</t>
+  </si>
+  <si>
+    <t>10P</t>
+  </si>
+  <si>
+    <t>12P</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>Prestige Elite</t>
+  </si>
+  <si>
+    <t>Essay</t>
+  </si>
+  <si>
+    <t>Courier</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>085</t>
+  </si>
+  <si>
+    <t>160</t>
+  </si>
+  <si>
+    <t>086</t>
+  </si>
+  <si>
+    <t>DP PC</t>
+  </si>
+  <si>
+    <t>001-008</t>
+  </si>
+  <si>
+    <t>Keyboard ID</t>
+  </si>
+  <si>
+    <t>Pitch</t>
+  </si>
+  <si>
+    <t>Reorder No.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6371,6 +6697,32 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -6658,7 +7010,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -6783,6 +7135,42 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -8162,6 +8550,1750 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D641A5B-6097-40F4-BC2F-54676E4E0DEA}">
+  <dimension ref="A1:E102"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" style="46" customWidth="1"/>
+    <col min="2" max="3" width="15.7109375" style="46" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="53" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" style="46" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" style="46" customWidth="1"/>
+    <col min="7" max="8" width="11.140625" style="46" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="46"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="45" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="44" t="s">
+        <v>335</v>
+      </c>
+      <c r="B1" s="44" t="s">
+        <v>433</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>433</v>
+      </c>
+      <c r="D1" s="51" t="s">
+        <v>432</v>
+      </c>
+      <c r="E1" s="44" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="45" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="44"/>
+      <c r="B2" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>435</v>
+      </c>
+      <c r="D2" s="52" t="s">
+        <v>436</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="45" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="44" t="s">
+        <v>440</v>
+      </c>
+      <c r="B3" s="50">
+        <v>102103</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>439</v>
+      </c>
+      <c r="D3" s="52" t="s">
+        <v>439</v>
+      </c>
+      <c r="E3" s="49" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="45" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="44"/>
+      <c r="B4" s="50" t="s">
+        <v>438</v>
+      </c>
+      <c r="C4" s="49"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="49"/>
+    </row>
+    <row r="5" spans="1:5" s="45" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="44" t="s">
+        <v>441</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>428</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>429</v>
+      </c>
+      <c r="D5" s="51" t="s">
+        <v>430</v>
+      </c>
+      <c r="E5" s="44" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="45" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
+        <v>442</v>
+      </c>
+      <c r="B6" s="44">
+        <v>1353909</v>
+      </c>
+      <c r="C6" s="44">
+        <v>1353523</v>
+      </c>
+      <c r="D6" s="51">
+        <v>1353526</v>
+      </c>
+      <c r="E6" s="44">
+        <v>1353502</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="46">
+        <v>1</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>336</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>336</v>
+      </c>
+      <c r="D7" s="53" t="s">
+        <v>336</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="46">
+        <v>2</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>337</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>337</v>
+      </c>
+      <c r="D8" s="53" t="s">
+        <v>337</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="46">
+        <v>3</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>338</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>338</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="46">
+        <v>4</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>339</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>339</v>
+      </c>
+      <c r="D10" s="53" t="s">
+        <v>339</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="46">
+        <v>5</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="D11" s="53" t="s">
+        <v>340</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="46">
+        <v>6</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>351</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>351</v>
+      </c>
+      <c r="D12" s="53" t="s">
+        <v>351</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="46">
+        <v>7</v>
+      </c>
+      <c r="B13" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="D13" s="53" t="s">
+        <v>342</v>
+      </c>
+      <c r="E13" s="46" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="46">
+        <v>8</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>343</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>343</v>
+      </c>
+      <c r="D14" s="53" t="s">
+        <v>343</v>
+      </c>
+      <c r="E14" s="46" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="46">
+        <v>9</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="D15" s="53" t="s">
+        <v>344</v>
+      </c>
+      <c r="E15" s="46" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="46">
+        <v>10</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>345</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>345</v>
+      </c>
+      <c r="D16" s="53" t="s">
+        <v>345</v>
+      </c>
+      <c r="E16" s="46" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="46">
+        <v>11</v>
+      </c>
+      <c r="B17" s="46" t="s">
+        <v>346</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>346</v>
+      </c>
+      <c r="D17" s="53" t="s">
+        <v>346</v>
+      </c>
+      <c r="E17" s="46" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="46">
+        <v>12</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>347</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>347</v>
+      </c>
+      <c r="D18" s="53" t="s">
+        <v>347</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="46">
+        <v>13</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>348</v>
+      </c>
+      <c r="C19" s="46" t="s">
+        <v>348</v>
+      </c>
+      <c r="D19" s="53" t="s">
+        <v>348</v>
+      </c>
+      <c r="E19" s="46" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="46">
+        <v>14</v>
+      </c>
+      <c r="B20" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>349</v>
+      </c>
+      <c r="D20" s="53" t="s">
+        <v>349</v>
+      </c>
+      <c r="E20" s="46" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="46">
+        <v>15</v>
+      </c>
+      <c r="B21" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="C21" s="46" t="s">
+        <v>350</v>
+      </c>
+      <c r="D21" s="53" t="s">
+        <v>350</v>
+      </c>
+      <c r="E21" s="46" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="46">
+        <v>16</v>
+      </c>
+      <c r="B22" s="46" t="s">
+        <v>341</v>
+      </c>
+      <c r="C22" s="46" t="s">
+        <v>341</v>
+      </c>
+      <c r="D22" s="53" t="s">
+        <v>341</v>
+      </c>
+      <c r="E22" s="46" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="46">
+        <v>17</v>
+      </c>
+      <c r="B23" s="46" t="s">
+        <v>352</v>
+      </c>
+      <c r="C23" s="46" t="s">
+        <v>352</v>
+      </c>
+      <c r="D23" s="53" t="s">
+        <v>352</v>
+      </c>
+      <c r="E23" s="46" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="46">
+        <v>18</v>
+      </c>
+      <c r="B24" s="46" t="s">
+        <v>353</v>
+      </c>
+      <c r="C24" s="46" t="s">
+        <v>353</v>
+      </c>
+      <c r="D24" s="53" t="s">
+        <v>353</v>
+      </c>
+      <c r="E24" s="46" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="46">
+        <v>19</v>
+      </c>
+      <c r="B25" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="C25" s="46" t="s">
+        <v>354</v>
+      </c>
+      <c r="D25" s="53" t="s">
+        <v>354</v>
+      </c>
+      <c r="E25" s="46" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="46">
+        <v>20</v>
+      </c>
+      <c r="B26" s="46" t="s">
+        <v>355</v>
+      </c>
+      <c r="C26" s="46" t="s">
+        <v>355</v>
+      </c>
+      <c r="D26" s="53" t="s">
+        <v>355</v>
+      </c>
+      <c r="E26" s="46" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="46">
+        <v>21</v>
+      </c>
+      <c r="B27" s="47" t="s">
+        <v>356</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>356</v>
+      </c>
+      <c r="D27" s="53" t="s">
+        <v>356</v>
+      </c>
+      <c r="E27" s="46" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="46">
+        <v>22</v>
+      </c>
+      <c r="B28" s="47" t="s">
+        <v>357</v>
+      </c>
+      <c r="C28" s="47" t="s">
+        <v>357</v>
+      </c>
+      <c r="D28" s="54" t="s">
+        <v>357</v>
+      </c>
+      <c r="E28" s="47" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="46">
+        <v>23</v>
+      </c>
+      <c r="B29" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="C29" s="46" t="s">
+        <v>358</v>
+      </c>
+      <c r="D29" s="53" t="s">
+        <v>358</v>
+      </c>
+      <c r="E29" s="46" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="46">
+        <v>24</v>
+      </c>
+      <c r="B30" s="46" t="s">
+        <v>359</v>
+      </c>
+      <c r="C30" s="46" t="s">
+        <v>359</v>
+      </c>
+      <c r="D30" s="53" t="s">
+        <v>359</v>
+      </c>
+      <c r="E30" s="46" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="46">
+        <v>25</v>
+      </c>
+      <c r="B31" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="C31" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="D31" s="53" t="s">
+        <v>360</v>
+      </c>
+      <c r="E31" s="46" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="46">
+        <v>26</v>
+      </c>
+      <c r="B32" s="46" t="s">
+        <v>361</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>427</v>
+      </c>
+      <c r="D32" s="54" t="s">
+        <v>427</v>
+      </c>
+      <c r="E32" s="47" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="46">
+        <v>27</v>
+      </c>
+      <c r="B33" s="46" t="s">
+        <v>362</v>
+      </c>
+      <c r="C33" s="48" t="s">
+        <v>426</v>
+      </c>
+      <c r="D33" s="55" t="s">
+        <v>426</v>
+      </c>
+      <c r="E33" s="48" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="46">
+        <v>28</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>363</v>
+      </c>
+      <c r="C34" s="46" t="s">
+        <v>425</v>
+      </c>
+      <c r="D34" s="53" t="s">
+        <v>425</v>
+      </c>
+      <c r="E34" s="46" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="46">
+        <v>29</v>
+      </c>
+      <c r="B35" s="46" t="s">
+        <v>364</v>
+      </c>
+      <c r="C35" s="46" t="s">
+        <v>424</v>
+      </c>
+      <c r="D35" s="53" t="s">
+        <v>424</v>
+      </c>
+      <c r="E35" s="46" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="46">
+        <v>30</v>
+      </c>
+      <c r="B36" s="46" t="s">
+        <v>365</v>
+      </c>
+      <c r="C36" s="46" t="s">
+        <v>423</v>
+      </c>
+      <c r="D36" s="53" t="s">
+        <v>423</v>
+      </c>
+      <c r="E36" s="46" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="46">
+        <v>31</v>
+      </c>
+      <c r="B37" s="46" t="s">
+        <v>366</v>
+      </c>
+      <c r="C37" s="46" t="s">
+        <v>422</v>
+      </c>
+      <c r="D37" s="53" t="s">
+        <v>422</v>
+      </c>
+      <c r="E37" s="46" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="46">
+        <v>32</v>
+      </c>
+      <c r="B38" s="46" t="s">
+        <v>367</v>
+      </c>
+      <c r="C38" s="46" t="s">
+        <v>421</v>
+      </c>
+      <c r="D38" s="53" t="s">
+        <v>421</v>
+      </c>
+      <c r="E38" s="46" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="46">
+        <v>33</v>
+      </c>
+      <c r="B39" s="46" t="s">
+        <v>368</v>
+      </c>
+      <c r="C39" s="46" t="s">
+        <v>369</v>
+      </c>
+      <c r="D39" s="53" t="s">
+        <v>369</v>
+      </c>
+      <c r="E39" s="46" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="46">
+        <v>34</v>
+      </c>
+      <c r="B40" s="46" t="s">
+        <v>369</v>
+      </c>
+      <c r="C40" s="46" t="s">
+        <v>368</v>
+      </c>
+      <c r="D40" s="53" t="s">
+        <v>368</v>
+      </c>
+      <c r="E40" s="46" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="46">
+        <v>35</v>
+      </c>
+      <c r="B41" s="46" t="s">
+        <v>370</v>
+      </c>
+      <c r="C41" s="46" t="s">
+        <v>370</v>
+      </c>
+      <c r="D41" s="53" t="s">
+        <v>370</v>
+      </c>
+      <c r="E41" s="46" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="46">
+        <v>36</v>
+      </c>
+      <c r="B42" s="46" t="s">
+        <v>371</v>
+      </c>
+      <c r="C42" s="46" t="s">
+        <v>371</v>
+      </c>
+      <c r="D42" s="53" t="s">
+        <v>371</v>
+      </c>
+      <c r="E42" s="46" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="46">
+        <v>37</v>
+      </c>
+      <c r="B43" s="46" t="s">
+        <v>372</v>
+      </c>
+      <c r="C43" s="46" t="s">
+        <v>372</v>
+      </c>
+      <c r="D43" s="53" t="s">
+        <v>372</v>
+      </c>
+      <c r="E43" s="46" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="46">
+        <v>38</v>
+      </c>
+      <c r="B44" s="46" t="s">
+        <v>373</v>
+      </c>
+      <c r="C44" s="47" t="s">
+        <v>420</v>
+      </c>
+      <c r="D44" s="54" t="s">
+        <v>420</v>
+      </c>
+      <c r="E44" s="47" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="46">
+        <v>39</v>
+      </c>
+      <c r="B45" s="46" t="s">
+        <v>374</v>
+      </c>
+      <c r="C45" s="46" t="s">
+        <v>374</v>
+      </c>
+      <c r="D45" s="53" t="s">
+        <v>374</v>
+      </c>
+      <c r="E45" s="46" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="46">
+        <v>40</v>
+      </c>
+      <c r="B46" s="46" t="s">
+        <v>375</v>
+      </c>
+      <c r="C46" s="46" t="s">
+        <v>419</v>
+      </c>
+      <c r="D46" s="53" t="s">
+        <v>419</v>
+      </c>
+      <c r="E46" s="46" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="46">
+        <v>41</v>
+      </c>
+      <c r="B47" s="46" t="s">
+        <v>376</v>
+      </c>
+      <c r="C47" s="46" t="s">
+        <v>376</v>
+      </c>
+      <c r="D47" s="53" t="s">
+        <v>376</v>
+      </c>
+      <c r="E47" s="46" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="46">
+        <v>42</v>
+      </c>
+      <c r="B48" s="46" t="s">
+        <v>377</v>
+      </c>
+      <c r="C48" s="46" t="s">
+        <v>377</v>
+      </c>
+      <c r="D48" s="53" t="s">
+        <v>377</v>
+      </c>
+      <c r="E48" s="46" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="46">
+        <v>43</v>
+      </c>
+      <c r="B49" s="46" t="s">
+        <v>378</v>
+      </c>
+      <c r="C49" s="46" t="s">
+        <v>378</v>
+      </c>
+      <c r="D49" s="53" t="s">
+        <v>378</v>
+      </c>
+      <c r="E49" s="46" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="46">
+        <v>44</v>
+      </c>
+      <c r="B50" s="46" t="s">
+        <v>379</v>
+      </c>
+      <c r="C50" s="46" t="s">
+        <v>379</v>
+      </c>
+      <c r="D50" s="53" t="s">
+        <v>379</v>
+      </c>
+      <c r="E50" s="46" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="46">
+        <v>45</v>
+      </c>
+      <c r="B51" s="46">
+        <v>7</v>
+      </c>
+      <c r="C51" s="46">
+        <v>7</v>
+      </c>
+      <c r="D51" s="53">
+        <v>7</v>
+      </c>
+      <c r="E51" s="46">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="46">
+        <v>46</v>
+      </c>
+      <c r="B52" s="46">
+        <v>8</v>
+      </c>
+      <c r="C52" s="46">
+        <v>8</v>
+      </c>
+      <c r="D52" s="53">
+        <v>8</v>
+      </c>
+      <c r="E52" s="46">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="46">
+        <v>47</v>
+      </c>
+      <c r="B53" s="46">
+        <v>6</v>
+      </c>
+      <c r="C53" s="46">
+        <v>6</v>
+      </c>
+      <c r="D53" s="53">
+        <v>6</v>
+      </c>
+      <c r="E53" s="46">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="46">
+        <v>48</v>
+      </c>
+      <c r="B54" s="46">
+        <v>4</v>
+      </c>
+      <c r="C54" s="46">
+        <v>4</v>
+      </c>
+      <c r="D54" s="53">
+        <v>4</v>
+      </c>
+      <c r="E54" s="46">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="46">
+        <v>49</v>
+      </c>
+      <c r="B55" s="46">
+        <v>5</v>
+      </c>
+      <c r="C55" s="46">
+        <v>5</v>
+      </c>
+      <c r="D55" s="53">
+        <v>5</v>
+      </c>
+      <c r="E55" s="46">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="46">
+        <v>50</v>
+      </c>
+      <c r="B56" s="46">
+        <v>0</v>
+      </c>
+      <c r="C56" s="46">
+        <v>0</v>
+      </c>
+      <c r="D56" s="53">
+        <v>0</v>
+      </c>
+      <c r="E56" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="46">
+        <v>51</v>
+      </c>
+      <c r="B57" s="46">
+        <v>2</v>
+      </c>
+      <c r="C57" s="46">
+        <v>2</v>
+      </c>
+      <c r="D57" s="53">
+        <v>2</v>
+      </c>
+      <c r="E57" s="46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="46">
+        <v>52</v>
+      </c>
+      <c r="B58" s="46">
+        <v>1</v>
+      </c>
+      <c r="C58" s="46">
+        <v>1</v>
+      </c>
+      <c r="D58" s="53">
+        <v>1</v>
+      </c>
+      <c r="E58" s="46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="46">
+        <v>53</v>
+      </c>
+      <c r="B59" s="46" t="s">
+        <v>380</v>
+      </c>
+      <c r="C59" s="46" t="s">
+        <v>380</v>
+      </c>
+      <c r="D59" s="53" t="s">
+        <v>380</v>
+      </c>
+      <c r="E59" s="46" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="46">
+        <v>54</v>
+      </c>
+      <c r="B60" s="46">
+        <v>3</v>
+      </c>
+      <c r="C60" s="46">
+        <v>3</v>
+      </c>
+      <c r="D60" s="53">
+        <v>3</v>
+      </c>
+      <c r="E60" s="46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="46">
+        <v>55</v>
+      </c>
+      <c r="B61" s="46" t="s">
+        <v>381</v>
+      </c>
+      <c r="C61" s="46" t="s">
+        <v>381</v>
+      </c>
+      <c r="D61" s="53" t="s">
+        <v>381</v>
+      </c>
+      <c r="E61" s="46" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="46">
+        <v>56</v>
+      </c>
+      <c r="B62" s="46">
+        <v>9</v>
+      </c>
+      <c r="C62" s="46">
+        <v>9</v>
+      </c>
+      <c r="D62" s="53">
+        <v>9</v>
+      </c>
+      <c r="E62" s="46">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="46">
+        <v>57</v>
+      </c>
+      <c r="B63" s="46" t="s">
+        <v>382</v>
+      </c>
+      <c r="C63" s="46" t="s">
+        <v>382</v>
+      </c>
+      <c r="D63" s="53" t="s">
+        <v>382</v>
+      </c>
+      <c r="E63" s="46" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="46">
+        <v>58</v>
+      </c>
+      <c r="B64" s="47" t="s">
+        <v>418</v>
+      </c>
+      <c r="C64" s="47" t="s">
+        <v>418</v>
+      </c>
+      <c r="D64" s="54" t="s">
+        <v>418</v>
+      </c>
+      <c r="E64" s="47" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="46">
+        <v>59</v>
+      </c>
+      <c r="B65" s="46" t="s">
+        <v>383</v>
+      </c>
+      <c r="C65" s="46" t="s">
+        <v>383</v>
+      </c>
+      <c r="D65" s="53" t="s">
+        <v>383</v>
+      </c>
+      <c r="E65" s="46" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="46">
+        <v>60</v>
+      </c>
+      <c r="B66" s="46" t="s">
+        <v>384</v>
+      </c>
+      <c r="C66" s="46" t="s">
+        <v>384</v>
+      </c>
+      <c r="D66" s="53" t="s">
+        <v>384</v>
+      </c>
+      <c r="E66" s="46" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="46">
+        <v>61</v>
+      </c>
+      <c r="B67" s="46" t="s">
+        <v>346</v>
+      </c>
+      <c r="C67" s="46" t="s">
+        <v>346</v>
+      </c>
+      <c r="D67" s="53" t="s">
+        <v>346</v>
+      </c>
+      <c r="E67" s="46" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="46">
+        <v>62</v>
+      </c>
+      <c r="B68" s="46" t="s">
+        <v>385</v>
+      </c>
+      <c r="C68" s="46" t="s">
+        <v>385</v>
+      </c>
+      <c r="D68" s="53" t="s">
+        <v>385</v>
+      </c>
+      <c r="E68" s="46" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="46">
+        <v>63</v>
+      </c>
+      <c r="B69" s="46" t="s">
+        <v>386</v>
+      </c>
+      <c r="C69" s="46" t="s">
+        <v>386</v>
+      </c>
+      <c r="D69" s="53" t="s">
+        <v>386</v>
+      </c>
+      <c r="E69" s="46" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="46">
+        <v>64</v>
+      </c>
+      <c r="B70" s="46" t="s">
+        <v>387</v>
+      </c>
+      <c r="C70" s="46" t="s">
+        <v>387</v>
+      </c>
+      <c r="D70" s="53" t="s">
+        <v>387</v>
+      </c>
+      <c r="E70" s="46" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="46">
+        <v>65</v>
+      </c>
+      <c r="B71" s="46" t="s">
+        <v>388</v>
+      </c>
+      <c r="C71" s="46" t="s">
+        <v>388</v>
+      </c>
+      <c r="D71" s="53" t="s">
+        <v>388</v>
+      </c>
+      <c r="E71" s="46" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="46">
+        <v>66</v>
+      </c>
+      <c r="B72" s="46" t="s">
+        <v>389</v>
+      </c>
+      <c r="C72" s="46" t="s">
+        <v>389</v>
+      </c>
+      <c r="D72" s="53" t="s">
+        <v>389</v>
+      </c>
+      <c r="E72" s="46" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="46">
+        <v>67</v>
+      </c>
+      <c r="B73" s="46" t="s">
+        <v>390</v>
+      </c>
+      <c r="C73" s="46" t="s">
+        <v>390</v>
+      </c>
+      <c r="D73" s="53" t="s">
+        <v>390</v>
+      </c>
+      <c r="E73" s="46" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="46">
+        <v>68</v>
+      </c>
+      <c r="B74" s="46" t="s">
+        <v>391</v>
+      </c>
+      <c r="C74" s="46" t="s">
+        <v>391</v>
+      </c>
+      <c r="D74" s="53" t="s">
+        <v>391</v>
+      </c>
+      <c r="E74" s="46" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="46">
+        <v>69</v>
+      </c>
+      <c r="B75" s="46" t="s">
+        <v>392</v>
+      </c>
+      <c r="C75" s="46" t="s">
+        <v>392</v>
+      </c>
+      <c r="D75" s="53" t="s">
+        <v>392</v>
+      </c>
+      <c r="E75" s="46" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="46">
+        <v>70</v>
+      </c>
+      <c r="B76" s="46" t="s">
+        <v>393</v>
+      </c>
+      <c r="C76" s="46" t="s">
+        <v>393</v>
+      </c>
+      <c r="D76" s="53" t="s">
+        <v>393</v>
+      </c>
+      <c r="E76" s="46" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="46">
+        <v>71</v>
+      </c>
+      <c r="B77" s="46" t="s">
+        <v>394</v>
+      </c>
+      <c r="C77" s="46" t="s">
+        <v>394</v>
+      </c>
+      <c r="D77" s="53" t="s">
+        <v>394</v>
+      </c>
+      <c r="E77" s="46" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="46">
+        <v>72</v>
+      </c>
+      <c r="B78" s="46" t="s">
+        <v>395</v>
+      </c>
+      <c r="C78" s="46" t="s">
+        <v>395</v>
+      </c>
+      <c r="D78" s="53" t="s">
+        <v>395</v>
+      </c>
+      <c r="E78" s="46" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="46">
+        <v>73</v>
+      </c>
+      <c r="B79" s="46" t="s">
+        <v>396</v>
+      </c>
+      <c r="C79" s="46" t="s">
+        <v>396</v>
+      </c>
+      <c r="D79" s="53" t="s">
+        <v>396</v>
+      </c>
+      <c r="E79" s="46" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="46">
+        <v>74</v>
+      </c>
+      <c r="B80" s="46" t="s">
+        <v>397</v>
+      </c>
+      <c r="C80" s="46" t="s">
+        <v>397</v>
+      </c>
+      <c r="D80" s="53" t="s">
+        <v>397</v>
+      </c>
+      <c r="E80" s="46" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="46">
+        <v>75</v>
+      </c>
+      <c r="B81" s="46" t="s">
+        <v>398</v>
+      </c>
+      <c r="C81" s="46" t="s">
+        <v>398</v>
+      </c>
+      <c r="D81" s="53" t="s">
+        <v>398</v>
+      </c>
+      <c r="E81" s="46" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="46">
+        <v>76</v>
+      </c>
+      <c r="B82" s="46" t="s">
+        <v>399</v>
+      </c>
+      <c r="C82" s="46" t="s">
+        <v>399</v>
+      </c>
+      <c r="D82" s="53" t="s">
+        <v>399</v>
+      </c>
+      <c r="E82" s="46" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="46">
+        <v>77</v>
+      </c>
+      <c r="B83" s="46" t="s">
+        <v>400</v>
+      </c>
+      <c r="C83" s="46" t="s">
+        <v>400</v>
+      </c>
+      <c r="D83" s="53" t="s">
+        <v>400</v>
+      </c>
+      <c r="E83" s="46" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="46">
+        <v>78</v>
+      </c>
+      <c r="B84" s="46" t="s">
+        <v>401</v>
+      </c>
+      <c r="C84" s="46" t="s">
+        <v>401</v>
+      </c>
+      <c r="D84" s="53" t="s">
+        <v>401</v>
+      </c>
+      <c r="E84" s="46" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="46">
+        <v>79</v>
+      </c>
+      <c r="B85" s="46" t="s">
+        <v>402</v>
+      </c>
+      <c r="C85" s="46" t="s">
+        <v>402</v>
+      </c>
+      <c r="D85" s="53" t="s">
+        <v>402</v>
+      </c>
+      <c r="E85" s="46" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="46">
+        <v>80</v>
+      </c>
+      <c r="B86" s="46" t="s">
+        <v>403</v>
+      </c>
+      <c r="C86" s="46" t="s">
+        <v>403</v>
+      </c>
+      <c r="D86" s="53" t="s">
+        <v>403</v>
+      </c>
+      <c r="E86" s="46" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="46">
+        <v>81</v>
+      </c>
+      <c r="B87" s="46" t="s">
+        <v>404</v>
+      </c>
+      <c r="C87" s="46" t="s">
+        <v>404</v>
+      </c>
+      <c r="D87" s="53" t="s">
+        <v>404</v>
+      </c>
+      <c r="E87" s="46" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="46">
+        <v>82</v>
+      </c>
+      <c r="B88" s="46" t="s">
+        <v>405</v>
+      </c>
+      <c r="C88" s="46" t="s">
+        <v>405</v>
+      </c>
+      <c r="D88" s="53" t="s">
+        <v>405</v>
+      </c>
+      <c r="E88" s="46" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="46">
+        <v>83</v>
+      </c>
+      <c r="B89" s="46" t="s">
+        <v>406</v>
+      </c>
+      <c r="C89" s="46" t="s">
+        <v>406</v>
+      </c>
+      <c r="D89" s="53" t="s">
+        <v>406</v>
+      </c>
+      <c r="E89" s="46" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" s="46">
+        <v>84</v>
+      </c>
+      <c r="B90" s="46" t="s">
+        <v>407</v>
+      </c>
+      <c r="C90" s="46" t="s">
+        <v>407</v>
+      </c>
+      <c r="D90" s="53" t="s">
+        <v>407</v>
+      </c>
+      <c r="E90" s="46" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" s="46">
+        <v>85</v>
+      </c>
+      <c r="B91" s="46" t="s">
+        <v>408</v>
+      </c>
+      <c r="C91" s="46" t="s">
+        <v>408</v>
+      </c>
+      <c r="D91" s="53" t="s">
+        <v>408</v>
+      </c>
+      <c r="E91" s="46" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="46">
+        <v>86</v>
+      </c>
+      <c r="B92" s="46" t="s">
+        <v>383</v>
+      </c>
+      <c r="C92" s="46" t="s">
+        <v>383</v>
+      </c>
+      <c r="D92" s="53" t="s">
+        <v>383</v>
+      </c>
+      <c r="E92" s="46" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="46">
+        <v>87</v>
+      </c>
+      <c r="B93" s="46" t="s">
+        <v>409</v>
+      </c>
+      <c r="C93" s="46" t="s">
+        <v>409</v>
+      </c>
+      <c r="D93" s="53" t="s">
+        <v>409</v>
+      </c>
+      <c r="E93" s="46" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" s="46">
+        <v>88</v>
+      </c>
+      <c r="B94" s="46" t="s">
+        <v>410</v>
+      </c>
+      <c r="C94" s="46" t="s">
+        <v>410</v>
+      </c>
+      <c r="D94" s="53" t="s">
+        <v>410</v>
+      </c>
+      <c r="E94" s="46" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" s="46">
+        <v>89</v>
+      </c>
+      <c r="B95" s="46" t="s">
+        <v>411</v>
+      </c>
+      <c r="C95" s="46" t="s">
+        <v>411</v>
+      </c>
+      <c r="D95" s="53" t="s">
+        <v>411</v>
+      </c>
+      <c r="E95" s="46" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="46">
+        <v>90</v>
+      </c>
+      <c r="B96" s="46" t="s">
+        <v>412</v>
+      </c>
+      <c r="C96" s="46" t="s">
+        <v>412</v>
+      </c>
+      <c r="D96" s="53" t="s">
+        <v>412</v>
+      </c>
+      <c r="E96" s="46" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" s="46">
+        <v>91</v>
+      </c>
+      <c r="B97" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="C97" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="D97" s="53" t="s">
+        <v>344</v>
+      </c>
+      <c r="E97" s="46" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" s="46">
+        <v>92</v>
+      </c>
+      <c r="B98" s="46" t="s">
+        <v>413</v>
+      </c>
+      <c r="C98" s="46" t="s">
+        <v>413</v>
+      </c>
+      <c r="D98" s="53" t="s">
+        <v>413</v>
+      </c>
+      <c r="E98" s="46" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" s="46">
+        <v>93</v>
+      </c>
+      <c r="B99" s="46" t="s">
+        <v>414</v>
+      </c>
+      <c r="C99" s="46" t="s">
+        <v>414</v>
+      </c>
+      <c r="D99" s="53" t="s">
+        <v>414</v>
+      </c>
+      <c r="E99" s="46" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" s="46">
+        <v>94</v>
+      </c>
+      <c r="B100" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="C100" s="46" t="s">
+        <v>415</v>
+      </c>
+      <c r="D100" s="53" t="s">
+        <v>415</v>
+      </c>
+      <c r="E100" s="46" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" s="46">
+        <v>95</v>
+      </c>
+      <c r="B101" s="46" t="s">
+        <v>416</v>
+      </c>
+      <c r="C101" s="46" t="s">
+        <v>416</v>
+      </c>
+      <c r="D101" s="53" t="s">
+        <v>416</v>
+      </c>
+      <c r="E101" s="46" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" s="46">
+        <v>96</v>
+      </c>
+      <c r="B102" s="46" t="s">
+        <v>417</v>
+      </c>
+      <c r="C102" s="46" t="s">
+        <v>417</v>
+      </c>
+      <c r="D102" s="53" t="s">
+        <v>417</v>
+      </c>
+      <c r="E102" s="46" t="s">
+        <v>417</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CBE5D03-400C-4374-BC8E-973FA89582E6}">
   <sheetPr>

</xml_diff>